<commit_message>
Statement template: right-to-left reading order in every text cell
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRrkjgeBdg5tEzYcZypdfp
</commit_message>
<xml_diff>
--- a/public/templates/statement-template.xlsx
+++ b/public/templates/statement-template.xlsx
@@ -184,67 +184,71 @@
   <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -621,7 +625,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">

</xml_diff>

<commit_message>
Statement template: generic filled example sheet (never imported)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GRrkjgeBdg5tEzYcZypdfp
</commit_message>
<xml_diff>
--- a/public/templates/statement-template.xlsx
+++ b/public/templates/statement-template.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="صورت وضعیت پروژه" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ریزمتر" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="نمونهٔ پرشده" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ریزمتر" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +92,12 @@
       <b val="1"/>
       <color rgb="000B1F3A"/>
       <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <b val="1"/>
+      <color rgb="008A6414"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -181,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -229,6 +236,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1373,6 +1383,914 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C8A24A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:H50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="B1" s="19" t="inlineStr">
+        <is>
+          <t>نمونهٔ پرشده — فقط برای دیدن؛ فرم خودتان را در برگهٔ «صورت وضعیت پروژه» پر کنید</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>نام پروژه :</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>پروژهٔ نمونه</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>شماره قرارداد :</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>NM-1405-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>موضوع قرارداد :</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>تهیه و نصب نمای آلومینیومی ساختمان نمونه</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>تاریخ قرارداد :</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>1405/01/15</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>(مثلاً ۱۴۰۵/۰۲/۰۶)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>کارفرما :</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>شرکت کارفرمای نمونه</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>نام پیمانکار</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>شرکت</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>(نام شرکت پیمانکار)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>شرکت پیمانکار نمونه</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>شماره آیتم قرارداد</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>شرح آیتم قرارداد</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>نوع</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>مقدار</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>واحد</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>فی</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>مبلغ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>تهیه و ساخت پنجره لولایی و فیکس</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>فروش / تأمین</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>مترمربع</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="H9" s="14">
+        <f>IF(OR(E9="",G9=""),"",E9*G9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>فروش لوور آلومینیومی</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>فروش / تأمین</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>مترطول</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="H10" s="14">
+        <f>IF(OR(E10="",G10=""),"",E10*G10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>فروش زیرسازی آلومینیومی نمای سنگی</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>فروش / تأمین</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>مترمربع</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="H11" s="14">
+        <f>IF(OR(E11="",G11=""),"",E11*G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>نصب پنجره لولایی و فیکس</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>نصب (مشمول بیمه)</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>مترمربع</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="H12" s="14">
+        <f>IF(OR(E12="",G12=""),"",E12*G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>نصب و اجرای لوور آلومینیومی</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>نصب (مشمول بیمه)</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>400</v>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>مترطول</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="H13" s="14">
+        <f>IF(OR(E13="",G13=""),"",E13*G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>نصب زیرسازی نمای سنگی</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>نصب (مشمول بیمه)</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>مترمربع</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="H14" s="14">
+        <f>IF(OR(E14="",G14=""),"",E14*G14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="14">
+        <f>IF(OR(E15="",G15=""),"",E15*G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="14">
+        <f>IF(OR(E16="",G16=""),"",E16*G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="14">
+        <f>IF(OR(E17="",G17=""),"",E17*G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="14">
+        <f>IF(OR(E18="",G18=""),"",E18*G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="14">
+        <f>IF(OR(E19="",G19=""),"",E19*G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="14">
+        <f>IF(OR(E20="",G20=""),"",E20*G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="14">
+        <f>IF(OR(E21="",G21=""),"",E21*G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="14">
+        <f>IF(OR(E22="",G22=""),"",E22*G22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="14">
+        <f>IF(OR(E23="",G23=""),"",E23*G23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="14">
+        <f>IF(OR(E24="",G24=""),"",E24*G24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="14">
+        <f>IF(OR(E25="",G25=""),"",E25*G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="14">
+        <f>IF(OR(E26="",G26=""),"",E26*G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="14">
+        <f>IF(OR(E27="",G27=""),"",E27*G27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="14">
+        <f>IF(OR(E28="",G28=""),"",E28*G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="14">
+        <f>IF(OR(E29="",G29=""),"",E29*G29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="14">
+        <f>IF(OR(E30="",G30=""),"",E30*G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="14">
+        <f>IF(OR(E31="",G31=""),"",E31*G31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C32" s="3" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="14">
+        <f>IF(OR(E32="",G32=""),"",E32*G32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="14">
+        <f>IF(OR(E33="",G33=""),"",E33*G33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="11" t="n"/>
+      <c r="G34" s="13" t="n"/>
+      <c r="H34" s="14">
+        <f>IF(OR(E34="",G34=""),"",E34*G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="13" t="n"/>
+      <c r="H35" s="14">
+        <f>IF(OR(E35="",G35=""),"",E35*G35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="13" t="n"/>
+      <c r="H36" s="14">
+        <f>IF(OR(E36="",G36=""),"",E36*G36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="13" t="n"/>
+      <c r="H37" s="14">
+        <f>IF(OR(E37="",G37=""),"",E37*G37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="14">
+        <f>IF(OR(E38="",G38=""),"",E38*G38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (1)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>مازاد نصب زیرسازی نمای سنگی</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>نصب (مشمول بیمه)</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>مترمربع</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="H39" s="14">
+        <f>IF(OR(E39="",G39=""),"",E39*G39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (2)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>جرثقیل</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>سایر</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>عدد</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="H40" s="14">
+        <f>IF(OR(E40="",G40=""),"",E40*G40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (3)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="13" t="n"/>
+      <c r="H41" s="14">
+        <f>IF(OR(E41="",G41=""),"",E41*G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (4)</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="13" t="n"/>
+      <c r="H42" s="14">
+        <f>IF(OR(E42="",G42=""),"",E42*G42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (5)</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="13" t="n"/>
+      <c r="H43" s="14">
+        <f>IF(OR(E43="",G43=""),"",E43*G43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (6)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="11" t="n"/>
+      <c r="G44" s="13" t="n"/>
+      <c r="H44" s="14">
+        <f>IF(OR(E44="",G44=""),"",E44*G44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (7)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="13" t="n"/>
+      <c r="H45" s="14">
+        <f>IF(OR(E45="",G45=""),"",E45*G45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (8)</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="11" t="n"/>
+      <c r="G46" s="13" t="n"/>
+      <c r="H46" s="14">
+        <f>IF(OR(E46="",G46=""),"",E46*G46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (9)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="13" t="n"/>
+      <c r="H47" s="14">
+        <f>IF(OR(E47="",G47=""),"",E47*G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>مازاد بر قرارداد (10)</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="13" t="n"/>
+      <c r="H48" s="14">
+        <f>IF(OR(E48="",G48=""),"",E48*G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>جمع کل</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="n"/>
+      <c r="D49" s="16" t="n"/>
+      <c r="E49" s="16" t="n"/>
+      <c r="F49" s="16" t="n"/>
+      <c r="G49" s="17">
+        <f>SUMPRODUCT(--(LEFT(B9:B48,5)&lt;&gt;"مازاد"),H9:H48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>تخفیف</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="n"/>
+      <c r="D50" s="16" t="n"/>
+      <c r="E50" s="16" t="n"/>
+      <c r="F50" s="16" t="n"/>
+      <c r="G50" s="18" t="n">
+        <v>1200000000</v>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>← مبلغ تخفیف کل قرارداد (اختیاری، ریال)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B49:F49"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1390,19 +2308,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>ریزمتره (اختیاری — مقدار انجام‌شدهٔ هر آیتم در هر صورت وضعیت)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>دوره کارکرد :</t>
         </is>
       </c>
-      <c r="B3" s="21" t="n"/>
+      <c r="B3" s="22" t="n"/>
       <c r="C3" s="5" t="n"/>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -1456,7 +2374,7 @@
       <c r="A6" s="11" t="n"/>
       <c r="B6" s="11" t="n"/>
       <c r="C6" s="11" t="n"/>
-      <c r="D6" s="22">
+      <c r="D6" s="23">
         <f>IF(A6="","",IFERROR(VLOOKUP(A6,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1475,7 +2393,7 @@
       <c r="A7" s="11" t="n"/>
       <c r="B7" s="11" t="n"/>
       <c r="C7" s="11" t="n"/>
-      <c r="D7" s="22">
+      <c r="D7" s="23">
         <f>IF(A7="","",IFERROR(VLOOKUP(A7,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1494,7 +2412,7 @@
       <c r="A8" s="11" t="n"/>
       <c r="B8" s="11" t="n"/>
       <c r="C8" s="11" t="n"/>
-      <c r="D8" s="22">
+      <c r="D8" s="23">
         <f>IF(A8="","",IFERROR(VLOOKUP(A8,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1513,7 +2431,7 @@
       <c r="A9" s="11" t="n"/>
       <c r="B9" s="11" t="n"/>
       <c r="C9" s="11" t="n"/>
-      <c r="D9" s="22">
+      <c r="D9" s="23">
         <f>IF(A9="","",IFERROR(VLOOKUP(A9,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1532,7 +2450,7 @@
       <c r="A10" s="11" t="n"/>
       <c r="B10" s="11" t="n"/>
       <c r="C10" s="11" t="n"/>
-      <c r="D10" s="22">
+      <c r="D10" s="23">
         <f>IF(A10="","",IFERROR(VLOOKUP(A10,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1551,7 +2469,7 @@
       <c r="A11" s="11" t="n"/>
       <c r="B11" s="11" t="n"/>
       <c r="C11" s="11" t="n"/>
-      <c r="D11" s="22">
+      <c r="D11" s="23">
         <f>IF(A11="","",IFERROR(VLOOKUP(A11,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1570,7 +2488,7 @@
       <c r="A12" s="11" t="n"/>
       <c r="B12" s="11" t="n"/>
       <c r="C12" s="11" t="n"/>
-      <c r="D12" s="22">
+      <c r="D12" s="23">
         <f>IF(A12="","",IFERROR(VLOOKUP(A12,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1589,7 +2507,7 @@
       <c r="A13" s="11" t="n"/>
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
-      <c r="D13" s="22">
+      <c r="D13" s="23">
         <f>IF(A13="","",IFERROR(VLOOKUP(A13,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1608,7 +2526,7 @@
       <c r="A14" s="11" t="n"/>
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
-      <c r="D14" s="22">
+      <c r="D14" s="23">
         <f>IF(A14="","",IFERROR(VLOOKUP(A14,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1627,7 +2545,7 @@
       <c r="A15" s="11" t="n"/>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="11" t="n"/>
-      <c r="D15" s="22">
+      <c r="D15" s="23">
         <f>IF(A15="","",IFERROR(VLOOKUP(A15,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1646,7 +2564,7 @@
       <c r="A16" s="11" t="n"/>
       <c r="B16" s="11" t="n"/>
       <c r="C16" s="11" t="n"/>
-      <c r="D16" s="22">
+      <c r="D16" s="23">
         <f>IF(A16="","",IFERROR(VLOOKUP(A16,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1665,7 +2583,7 @@
       <c r="A17" s="11" t="n"/>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="11" t="n"/>
-      <c r="D17" s="22">
+      <c r="D17" s="23">
         <f>IF(A17="","",IFERROR(VLOOKUP(A17,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1684,7 +2602,7 @@
       <c r="A18" s="11" t="n"/>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
-      <c r="D18" s="22">
+      <c r="D18" s="23">
         <f>IF(A18="","",IFERROR(VLOOKUP(A18,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1703,7 +2621,7 @@
       <c r="A19" s="11" t="n"/>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
-      <c r="D19" s="22">
+      <c r="D19" s="23">
         <f>IF(A19="","",IFERROR(VLOOKUP(A19,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1722,7 +2640,7 @@
       <c r="A20" s="11" t="n"/>
       <c r="B20" s="11" t="n"/>
       <c r="C20" s="11" t="n"/>
-      <c r="D20" s="22">
+      <c r="D20" s="23">
         <f>IF(A20="","",IFERROR(VLOOKUP(A20,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1741,7 +2659,7 @@
       <c r="A21" s="11" t="n"/>
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="11" t="n"/>
-      <c r="D21" s="22">
+      <c r="D21" s="23">
         <f>IF(A21="","",IFERROR(VLOOKUP(A21,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1760,7 +2678,7 @@
       <c r="A22" s="11" t="n"/>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="11" t="n"/>
-      <c r="D22" s="22">
+      <c r="D22" s="23">
         <f>IF(A22="","",IFERROR(VLOOKUP(A22,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1779,7 +2697,7 @@
       <c r="A23" s="11" t="n"/>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="11" t="n"/>
-      <c r="D23" s="22">
+      <c r="D23" s="23">
         <f>IF(A23="","",IFERROR(VLOOKUP(A23,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1798,7 +2716,7 @@
       <c r="A24" s="11" t="n"/>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="11" t="n"/>
-      <c r="D24" s="22">
+      <c r="D24" s="23">
         <f>IF(A24="","",IFERROR(VLOOKUP(A24,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1817,7 +2735,7 @@
       <c r="A25" s="11" t="n"/>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
-      <c r="D25" s="22">
+      <c r="D25" s="23">
         <f>IF(A25="","",IFERROR(VLOOKUP(A25,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1836,7 +2754,7 @@
       <c r="A26" s="11" t="n"/>
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
-      <c r="D26" s="22">
+      <c r="D26" s="23">
         <f>IF(A26="","",IFERROR(VLOOKUP(A26,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1855,7 +2773,7 @@
       <c r="A27" s="11" t="n"/>
       <c r="B27" s="11" t="n"/>
       <c r="C27" s="11" t="n"/>
-      <c r="D27" s="22">
+      <c r="D27" s="23">
         <f>IF(A27="","",IFERROR(VLOOKUP(A27,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1874,7 +2792,7 @@
       <c r="A28" s="11" t="n"/>
       <c r="B28" s="11" t="n"/>
       <c r="C28" s="11" t="n"/>
-      <c r="D28" s="22">
+      <c r="D28" s="23">
         <f>IF(A28="","",IFERROR(VLOOKUP(A28,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1893,7 +2811,7 @@
       <c r="A29" s="11" t="n"/>
       <c r="B29" s="11" t="n"/>
       <c r="C29" s="11" t="n"/>
-      <c r="D29" s="22">
+      <c r="D29" s="23">
         <f>IF(A29="","",IFERROR(VLOOKUP(A29,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1912,7 +2830,7 @@
       <c r="A30" s="11" t="n"/>
       <c r="B30" s="11" t="n"/>
       <c r="C30" s="11" t="n"/>
-      <c r="D30" s="22">
+      <c r="D30" s="23">
         <f>IF(A30="","",IFERROR(VLOOKUP(A30,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1931,7 +2849,7 @@
       <c r="A31" s="11" t="n"/>
       <c r="B31" s="11" t="n"/>
       <c r="C31" s="11" t="n"/>
-      <c r="D31" s="22">
+      <c r="D31" s="23">
         <f>IF(A31="","",IFERROR(VLOOKUP(A31,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1950,7 +2868,7 @@
       <c r="A32" s="11" t="n"/>
       <c r="B32" s="11" t="n"/>
       <c r="C32" s="11" t="n"/>
-      <c r="D32" s="22">
+      <c r="D32" s="23">
         <f>IF(A32="","",IFERROR(VLOOKUP(A32,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1969,7 +2887,7 @@
       <c r="A33" s="11" t="n"/>
       <c r="B33" s="11" t="n"/>
       <c r="C33" s="11" t="n"/>
-      <c r="D33" s="22">
+      <c r="D33" s="23">
         <f>IF(A33="","",IFERROR(VLOOKUP(A33,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -1988,7 +2906,7 @@
       <c r="A34" s="11" t="n"/>
       <c r="B34" s="11" t="n"/>
       <c r="C34" s="11" t="n"/>
-      <c r="D34" s="22">
+      <c r="D34" s="23">
         <f>IF(A34="","",IFERROR(VLOOKUP(A34,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2007,7 +2925,7 @@
       <c r="A35" s="11" t="n"/>
       <c r="B35" s="11" t="n"/>
       <c r="C35" s="11" t="n"/>
-      <c r="D35" s="22">
+      <c r="D35" s="23">
         <f>IF(A35="","",IFERROR(VLOOKUP(A35,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2026,7 +2944,7 @@
       <c r="A36" s="11" t="n"/>
       <c r="B36" s="11" t="n"/>
       <c r="C36" s="11" t="n"/>
-      <c r="D36" s="22">
+      <c r="D36" s="23">
         <f>IF(A36="","",IFERROR(VLOOKUP(A36,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2045,7 +2963,7 @@
       <c r="A37" s="11" t="n"/>
       <c r="B37" s="11" t="n"/>
       <c r="C37" s="11" t="n"/>
-      <c r="D37" s="22">
+      <c r="D37" s="23">
         <f>IF(A37="","",IFERROR(VLOOKUP(A37,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2064,7 +2982,7 @@
       <c r="A38" s="11" t="n"/>
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="11" t="n"/>
-      <c r="D38" s="22">
+      <c r="D38" s="23">
         <f>IF(A38="","",IFERROR(VLOOKUP(A38,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2083,7 +3001,7 @@
       <c r="A39" s="11" t="n"/>
       <c r="B39" s="11" t="n"/>
       <c r="C39" s="11" t="n"/>
-      <c r="D39" s="22">
+      <c r="D39" s="23">
         <f>IF(A39="","",IFERROR(VLOOKUP(A39,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2102,7 +3020,7 @@
       <c r="A40" s="11" t="n"/>
       <c r="B40" s="11" t="n"/>
       <c r="C40" s="11" t="n"/>
-      <c r="D40" s="22">
+      <c r="D40" s="23">
         <f>IF(A40="","",IFERROR(VLOOKUP(A40,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2121,7 +3039,7 @@
       <c r="A41" s="11" t="n"/>
       <c r="B41" s="11" t="n"/>
       <c r="C41" s="11" t="n"/>
-      <c r="D41" s="22">
+      <c r="D41" s="23">
         <f>IF(A41="","",IFERROR(VLOOKUP(A41,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2140,7 +3058,7 @@
       <c r="A42" s="11" t="n"/>
       <c r="B42" s="11" t="n"/>
       <c r="C42" s="11" t="n"/>
-      <c r="D42" s="22">
+      <c r="D42" s="23">
         <f>IF(A42="","",IFERROR(VLOOKUP(A42,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2159,7 +3077,7 @@
       <c r="A43" s="11" t="n"/>
       <c r="B43" s="11" t="n"/>
       <c r="C43" s="11" t="n"/>
-      <c r="D43" s="22">
+      <c r="D43" s="23">
         <f>IF(A43="","",IFERROR(VLOOKUP(A43,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2178,7 +3096,7 @@
       <c r="A44" s="11" t="n"/>
       <c r="B44" s="11" t="n"/>
       <c r="C44" s="11" t="n"/>
-      <c r="D44" s="22">
+      <c r="D44" s="23">
         <f>IF(A44="","",IFERROR(VLOOKUP(A44,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2197,7 +3115,7 @@
       <c r="A45" s="11" t="n"/>
       <c r="B45" s="11" t="n"/>
       <c r="C45" s="11" t="n"/>
-      <c r="D45" s="22">
+      <c r="D45" s="23">
         <f>IF(A45="","",IFERROR(VLOOKUP(A45,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2216,7 +3134,7 @@
       <c r="A46" s="11" t="n"/>
       <c r="B46" s="11" t="n"/>
       <c r="C46" s="11" t="n"/>
-      <c r="D46" s="22">
+      <c r="D46" s="23">
         <f>IF(A46="","",IFERROR(VLOOKUP(A46,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2235,7 +3153,7 @@
       <c r="A47" s="11" t="n"/>
       <c r="B47" s="11" t="n"/>
       <c r="C47" s="11" t="n"/>
-      <c r="D47" s="22">
+      <c r="D47" s="23">
         <f>IF(A47="","",IFERROR(VLOOKUP(A47,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2254,7 +3172,7 @@
       <c r="A48" s="11" t="n"/>
       <c r="B48" s="11" t="n"/>
       <c r="C48" s="11" t="n"/>
-      <c r="D48" s="22">
+      <c r="D48" s="23">
         <f>IF(A48="","",IFERROR(VLOOKUP(A48,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2273,7 +3191,7 @@
       <c r="A49" s="11" t="n"/>
       <c r="B49" s="11" t="n"/>
       <c r="C49" s="11" t="n"/>
-      <c r="D49" s="22">
+      <c r="D49" s="23">
         <f>IF(A49="","",IFERROR(VLOOKUP(A49,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2292,7 +3210,7 @@
       <c r="A50" s="11" t="n"/>
       <c r="B50" s="11" t="n"/>
       <c r="C50" s="11" t="n"/>
-      <c r="D50" s="22">
+      <c r="D50" s="23">
         <f>IF(A50="","",IFERROR(VLOOKUP(A50,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2311,7 +3229,7 @@
       <c r="A51" s="11" t="n"/>
       <c r="B51" s="11" t="n"/>
       <c r="C51" s="11" t="n"/>
-      <c r="D51" s="22">
+      <c r="D51" s="23">
         <f>IF(A51="","",IFERROR(VLOOKUP(A51,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2330,7 +3248,7 @@
       <c r="A52" s="11" t="n"/>
       <c r="B52" s="11" t="n"/>
       <c r="C52" s="11" t="n"/>
-      <c r="D52" s="22">
+      <c r="D52" s="23">
         <f>IF(A52="","",IFERROR(VLOOKUP(A52,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2349,7 +3267,7 @@
       <c r="A53" s="11" t="n"/>
       <c r="B53" s="11" t="n"/>
       <c r="C53" s="11" t="n"/>
-      <c r="D53" s="22">
+      <c r="D53" s="23">
         <f>IF(A53="","",IFERROR(VLOOKUP(A53,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2368,7 +3286,7 @@
       <c r="A54" s="11" t="n"/>
       <c r="B54" s="11" t="n"/>
       <c r="C54" s="11" t="n"/>
-      <c r="D54" s="22">
+      <c r="D54" s="23">
         <f>IF(A54="","",IFERROR(VLOOKUP(A54,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2387,7 +3305,7 @@
       <c r="A55" s="11" t="n"/>
       <c r="B55" s="11" t="n"/>
       <c r="C55" s="11" t="n"/>
-      <c r="D55" s="22">
+      <c r="D55" s="23">
         <f>IF(A55="","",IFERROR(VLOOKUP(A55,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2406,7 +3324,7 @@
       <c r="A56" s="11" t="n"/>
       <c r="B56" s="11" t="n"/>
       <c r="C56" s="11" t="n"/>
-      <c r="D56" s="22">
+      <c r="D56" s="23">
         <f>IF(A56="","",IFERROR(VLOOKUP(A56,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2425,7 +3343,7 @@
       <c r="A57" s="11" t="n"/>
       <c r="B57" s="11" t="n"/>
       <c r="C57" s="11" t="n"/>
-      <c r="D57" s="22">
+      <c r="D57" s="23">
         <f>IF(A57="","",IFERROR(VLOOKUP(A57,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2444,7 +3362,7 @@
       <c r="A58" s="11" t="n"/>
       <c r="B58" s="11" t="n"/>
       <c r="C58" s="11" t="n"/>
-      <c r="D58" s="22">
+      <c r="D58" s="23">
         <f>IF(A58="","",IFERROR(VLOOKUP(A58,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2463,7 +3381,7 @@
       <c r="A59" s="11" t="n"/>
       <c r="B59" s="11" t="n"/>
       <c r="C59" s="11" t="n"/>
-      <c r="D59" s="22">
+      <c r="D59" s="23">
         <f>IF(A59="","",IFERROR(VLOOKUP(A59,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2482,7 +3400,7 @@
       <c r="A60" s="11" t="n"/>
       <c r="B60" s="11" t="n"/>
       <c r="C60" s="11" t="n"/>
-      <c r="D60" s="22">
+      <c r="D60" s="23">
         <f>IF(A60="","",IFERROR(VLOOKUP(A60,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2501,7 +3419,7 @@
       <c r="A61" s="11" t="n"/>
       <c r="B61" s="11" t="n"/>
       <c r="C61" s="11" t="n"/>
-      <c r="D61" s="22">
+      <c r="D61" s="23">
         <f>IF(A61="","",IFERROR(VLOOKUP(A61,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2520,7 +3438,7 @@
       <c r="A62" s="11" t="n"/>
       <c r="B62" s="11" t="n"/>
       <c r="C62" s="11" t="n"/>
-      <c r="D62" s="22">
+      <c r="D62" s="23">
         <f>IF(A62="","",IFERROR(VLOOKUP(A62,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2539,7 +3457,7 @@
       <c r="A63" s="11" t="n"/>
       <c r="B63" s="11" t="n"/>
       <c r="C63" s="11" t="n"/>
-      <c r="D63" s="22">
+      <c r="D63" s="23">
         <f>IF(A63="","",IFERROR(VLOOKUP(A63,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2558,7 +3476,7 @@
       <c r="A64" s="11" t="n"/>
       <c r="B64" s="11" t="n"/>
       <c r="C64" s="11" t="n"/>
-      <c r="D64" s="22">
+      <c r="D64" s="23">
         <f>IF(A64="","",IFERROR(VLOOKUP(A64,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2577,7 +3495,7 @@
       <c r="A65" s="11" t="n"/>
       <c r="B65" s="11" t="n"/>
       <c r="C65" s="11" t="n"/>
-      <c r="D65" s="22">
+      <c r="D65" s="23">
         <f>IF(A65="","",IFERROR(VLOOKUP(A65,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2596,7 +3514,7 @@
       <c r="A66" s="11" t="n"/>
       <c r="B66" s="11" t="n"/>
       <c r="C66" s="11" t="n"/>
-      <c r="D66" s="22">
+      <c r="D66" s="23">
         <f>IF(A66="","",IFERROR(VLOOKUP(A66,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2615,7 +3533,7 @@
       <c r="A67" s="11" t="n"/>
       <c r="B67" s="11" t="n"/>
       <c r="C67" s="11" t="n"/>
-      <c r="D67" s="22">
+      <c r="D67" s="23">
         <f>IF(A67="","",IFERROR(VLOOKUP(A67,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2634,7 +3552,7 @@
       <c r="A68" s="11" t="n"/>
       <c r="B68" s="11" t="n"/>
       <c r="C68" s="11" t="n"/>
-      <c r="D68" s="22">
+      <c r="D68" s="23">
         <f>IF(A68="","",IFERROR(VLOOKUP(A68,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2653,7 +3571,7 @@
       <c r="A69" s="11" t="n"/>
       <c r="B69" s="11" t="n"/>
       <c r="C69" s="11" t="n"/>
-      <c r="D69" s="22">
+      <c r="D69" s="23">
         <f>IF(A69="","",IFERROR(VLOOKUP(A69,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2672,7 +3590,7 @@
       <c r="A70" s="11" t="n"/>
       <c r="B70" s="11" t="n"/>
       <c r="C70" s="11" t="n"/>
-      <c r="D70" s="22">
+      <c r="D70" s="23">
         <f>IF(A70="","",IFERROR(VLOOKUP(A70,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2691,7 +3609,7 @@
       <c r="A71" s="11" t="n"/>
       <c r="B71" s="11" t="n"/>
       <c r="C71" s="11" t="n"/>
-      <c r="D71" s="22">
+      <c r="D71" s="23">
         <f>IF(A71="","",IFERROR(VLOOKUP(A71,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2710,7 +3628,7 @@
       <c r="A72" s="11" t="n"/>
       <c r="B72" s="11" t="n"/>
       <c r="C72" s="11" t="n"/>
-      <c r="D72" s="22">
+      <c r="D72" s="23">
         <f>IF(A72="","",IFERROR(VLOOKUP(A72,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2729,7 +3647,7 @@
       <c r="A73" s="11" t="n"/>
       <c r="B73" s="11" t="n"/>
       <c r="C73" s="11" t="n"/>
-      <c r="D73" s="22">
+      <c r="D73" s="23">
         <f>IF(A73="","",IFERROR(VLOOKUP(A73,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2748,7 +3666,7 @@
       <c r="A74" s="11" t="n"/>
       <c r="B74" s="11" t="n"/>
       <c r="C74" s="11" t="n"/>
-      <c r="D74" s="22">
+      <c r="D74" s="23">
         <f>IF(A74="","",IFERROR(VLOOKUP(A74,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2767,7 +3685,7 @@
       <c r="A75" s="11" t="n"/>
       <c r="B75" s="11" t="n"/>
       <c r="C75" s="11" t="n"/>
-      <c r="D75" s="22">
+      <c r="D75" s="23">
         <f>IF(A75="","",IFERROR(VLOOKUP(A75,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2786,7 +3704,7 @@
       <c r="A76" s="11" t="n"/>
       <c r="B76" s="11" t="n"/>
       <c r="C76" s="11" t="n"/>
-      <c r="D76" s="22">
+      <c r="D76" s="23">
         <f>IF(A76="","",IFERROR(VLOOKUP(A76,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2805,7 +3723,7 @@
       <c r="A77" s="11" t="n"/>
       <c r="B77" s="11" t="n"/>
       <c r="C77" s="11" t="n"/>
-      <c r="D77" s="22">
+      <c r="D77" s="23">
         <f>IF(A77="","",IFERROR(VLOOKUP(A77,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2824,7 +3742,7 @@
       <c r="A78" s="11" t="n"/>
       <c r="B78" s="11" t="n"/>
       <c r="C78" s="11" t="n"/>
-      <c r="D78" s="22">
+      <c r="D78" s="23">
         <f>IF(A78="","",IFERROR(VLOOKUP(A78,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2843,7 +3761,7 @@
       <c r="A79" s="11" t="n"/>
       <c r="B79" s="11" t="n"/>
       <c r="C79" s="11" t="n"/>
-      <c r="D79" s="22">
+      <c r="D79" s="23">
         <f>IF(A79="","",IFERROR(VLOOKUP(A79,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2862,7 +3780,7 @@
       <c r="A80" s="11" t="n"/>
       <c r="B80" s="11" t="n"/>
       <c r="C80" s="11" t="n"/>
-      <c r="D80" s="22">
+      <c r="D80" s="23">
         <f>IF(A80="","",IFERROR(VLOOKUP(A80,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2881,7 +3799,7 @@
       <c r="A81" s="11" t="n"/>
       <c r="B81" s="11" t="n"/>
       <c r="C81" s="11" t="n"/>
-      <c r="D81" s="22">
+      <c r="D81" s="23">
         <f>IF(A81="","",IFERROR(VLOOKUP(A81,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2900,7 +3818,7 @@
       <c r="A82" s="11" t="n"/>
       <c r="B82" s="11" t="n"/>
       <c r="C82" s="11" t="n"/>
-      <c r="D82" s="22">
+      <c r="D82" s="23">
         <f>IF(A82="","",IFERROR(VLOOKUP(A82,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2919,7 +3837,7 @@
       <c r="A83" s="11" t="n"/>
       <c r="B83" s="11" t="n"/>
       <c r="C83" s="11" t="n"/>
-      <c r="D83" s="22">
+      <c r="D83" s="23">
         <f>IF(A83="","",IFERROR(VLOOKUP(A83,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2938,7 +3856,7 @@
       <c r="A84" s="11" t="n"/>
       <c r="B84" s="11" t="n"/>
       <c r="C84" s="11" t="n"/>
-      <c r="D84" s="22">
+      <c r="D84" s="23">
         <f>IF(A84="","",IFERROR(VLOOKUP(A84,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2957,7 +3875,7 @@
       <c r="A85" s="11" t="n"/>
       <c r="B85" s="11" t="n"/>
       <c r="C85" s="11" t="n"/>
-      <c r="D85" s="22">
+      <c r="D85" s="23">
         <f>IF(A85="","",IFERROR(VLOOKUP(A85,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2976,7 +3894,7 @@
       <c r="A86" s="11" t="n"/>
       <c r="B86" s="11" t="n"/>
       <c r="C86" s="11" t="n"/>
-      <c r="D86" s="22">
+      <c r="D86" s="23">
         <f>IF(A86="","",IFERROR(VLOOKUP(A86,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -2995,7 +3913,7 @@
       <c r="A87" s="11" t="n"/>
       <c r="B87" s="11" t="n"/>
       <c r="C87" s="11" t="n"/>
-      <c r="D87" s="22">
+      <c r="D87" s="23">
         <f>IF(A87="","",IFERROR(VLOOKUP(A87,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3014,7 +3932,7 @@
       <c r="A88" s="11" t="n"/>
       <c r="B88" s="11" t="n"/>
       <c r="C88" s="11" t="n"/>
-      <c r="D88" s="22">
+      <c r="D88" s="23">
         <f>IF(A88="","",IFERROR(VLOOKUP(A88,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3033,7 +3951,7 @@
       <c r="A89" s="11" t="n"/>
       <c r="B89" s="11" t="n"/>
       <c r="C89" s="11" t="n"/>
-      <c r="D89" s="22">
+      <c r="D89" s="23">
         <f>IF(A89="","",IFERROR(VLOOKUP(A89,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3052,7 +3970,7 @@
       <c r="A90" s="11" t="n"/>
       <c r="B90" s="11" t="n"/>
       <c r="C90" s="11" t="n"/>
-      <c r="D90" s="22">
+      <c r="D90" s="23">
         <f>IF(A90="","",IFERROR(VLOOKUP(A90,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3071,7 +3989,7 @@
       <c r="A91" s="11" t="n"/>
       <c r="B91" s="11" t="n"/>
       <c r="C91" s="11" t="n"/>
-      <c r="D91" s="22">
+      <c r="D91" s="23">
         <f>IF(A91="","",IFERROR(VLOOKUP(A91,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3090,7 +4008,7 @@
       <c r="A92" s="11" t="n"/>
       <c r="B92" s="11" t="n"/>
       <c r="C92" s="11" t="n"/>
-      <c r="D92" s="22">
+      <c r="D92" s="23">
         <f>IF(A92="","",IFERROR(VLOOKUP(A92,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3109,7 +4027,7 @@
       <c r="A93" s="11" t="n"/>
       <c r="B93" s="11" t="n"/>
       <c r="C93" s="11" t="n"/>
-      <c r="D93" s="22">
+      <c r="D93" s="23">
         <f>IF(A93="","",IFERROR(VLOOKUP(A93,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3128,7 +4046,7 @@
       <c r="A94" s="11" t="n"/>
       <c r="B94" s="11" t="n"/>
       <c r="C94" s="11" t="n"/>
-      <c r="D94" s="22">
+      <c r="D94" s="23">
         <f>IF(A94="","",IFERROR(VLOOKUP(A94,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3147,7 +4065,7 @@
       <c r="A95" s="11" t="n"/>
       <c r="B95" s="11" t="n"/>
       <c r="C95" s="11" t="n"/>
-      <c r="D95" s="22">
+      <c r="D95" s="23">
         <f>IF(A95="","",IFERROR(VLOOKUP(A95,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3166,7 +4084,7 @@
       <c r="A96" s="11" t="n"/>
       <c r="B96" s="11" t="n"/>
       <c r="C96" s="11" t="n"/>
-      <c r="D96" s="22">
+      <c r="D96" s="23">
         <f>IF(A96="","",IFERROR(VLOOKUP(A96,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3185,7 +4103,7 @@
       <c r="A97" s="11" t="n"/>
       <c r="B97" s="11" t="n"/>
       <c r="C97" s="11" t="n"/>
-      <c r="D97" s="22">
+      <c r="D97" s="23">
         <f>IF(A97="","",IFERROR(VLOOKUP(A97,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3204,7 +4122,7 @@
       <c r="A98" s="11" t="n"/>
       <c r="B98" s="11" t="n"/>
       <c r="C98" s="11" t="n"/>
-      <c r="D98" s="22">
+      <c r="D98" s="23">
         <f>IF(A98="","",IFERROR(VLOOKUP(A98,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3223,7 +4141,7 @@
       <c r="A99" s="11" t="n"/>
       <c r="B99" s="11" t="n"/>
       <c r="C99" s="11" t="n"/>
-      <c r="D99" s="22">
+      <c r="D99" s="23">
         <f>IF(A99="","",IFERROR(VLOOKUP(A99,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3242,7 +4160,7 @@
       <c r="A100" s="11" t="n"/>
       <c r="B100" s="11" t="n"/>
       <c r="C100" s="11" t="n"/>
-      <c r="D100" s="22">
+      <c r="D100" s="23">
         <f>IF(A100="","",IFERROR(VLOOKUP(A100,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3261,7 +4179,7 @@
       <c r="A101" s="11" t="n"/>
       <c r="B101" s="11" t="n"/>
       <c r="C101" s="11" t="n"/>
-      <c r="D101" s="22">
+      <c r="D101" s="23">
         <f>IF(A101="","",IFERROR(VLOOKUP(A101,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3280,7 +4198,7 @@
       <c r="A102" s="11" t="n"/>
       <c r="B102" s="11" t="n"/>
       <c r="C102" s="11" t="n"/>
-      <c r="D102" s="22">
+      <c r="D102" s="23">
         <f>IF(A102="","",IFERROR(VLOOKUP(A102,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3299,7 +4217,7 @@
       <c r="A103" s="11" t="n"/>
       <c r="B103" s="11" t="n"/>
       <c r="C103" s="11" t="n"/>
-      <c r="D103" s="22">
+      <c r="D103" s="23">
         <f>IF(A103="","",IFERROR(VLOOKUP(A103,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3318,7 +4236,7 @@
       <c r="A104" s="11" t="n"/>
       <c r="B104" s="11" t="n"/>
       <c r="C104" s="11" t="n"/>
-      <c r="D104" s="22">
+      <c r="D104" s="23">
         <f>IF(A104="","",IFERROR(VLOOKUP(A104,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3337,7 +4255,7 @@
       <c r="A105" s="11" t="n"/>
       <c r="B105" s="11" t="n"/>
       <c r="C105" s="11" t="n"/>
-      <c r="D105" s="22">
+      <c r="D105" s="23">
         <f>IF(A105="","",IFERROR(VLOOKUP(A105,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3356,7 +4274,7 @@
       <c r="A106" s="11" t="n"/>
       <c r="B106" s="11" t="n"/>
       <c r="C106" s="11" t="n"/>
-      <c r="D106" s="22">
+      <c r="D106" s="23">
         <f>IF(A106="","",IFERROR(VLOOKUP(A106,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3375,7 +4293,7 @@
       <c r="A107" s="11" t="n"/>
       <c r="B107" s="11" t="n"/>
       <c r="C107" s="11" t="n"/>
-      <c r="D107" s="22">
+      <c r="D107" s="23">
         <f>IF(A107="","",IFERROR(VLOOKUP(A107,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3394,7 +4312,7 @@
       <c r="A108" s="11" t="n"/>
       <c r="B108" s="11" t="n"/>
       <c r="C108" s="11" t="n"/>
-      <c r="D108" s="22">
+      <c r="D108" s="23">
         <f>IF(A108="","",IFERROR(VLOOKUP(A108,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3413,7 +4331,7 @@
       <c r="A109" s="11" t="n"/>
       <c r="B109" s="11" t="n"/>
       <c r="C109" s="11" t="n"/>
-      <c r="D109" s="22">
+      <c r="D109" s="23">
         <f>IF(A109="","",IFERROR(VLOOKUP(A109,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3432,7 +4350,7 @@
       <c r="A110" s="11" t="n"/>
       <c r="B110" s="11" t="n"/>
       <c r="C110" s="11" t="n"/>
-      <c r="D110" s="22">
+      <c r="D110" s="23">
         <f>IF(A110="","",IFERROR(VLOOKUP(A110,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3451,7 +4369,7 @@
       <c r="A111" s="11" t="n"/>
       <c r="B111" s="11" t="n"/>
       <c r="C111" s="11" t="n"/>
-      <c r="D111" s="22">
+      <c r="D111" s="23">
         <f>IF(A111="","",IFERROR(VLOOKUP(A111,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3470,7 +4388,7 @@
       <c r="A112" s="11" t="n"/>
       <c r="B112" s="11" t="n"/>
       <c r="C112" s="11" t="n"/>
-      <c r="D112" s="22">
+      <c r="D112" s="23">
         <f>IF(A112="","",IFERROR(VLOOKUP(A112,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3489,7 +4407,7 @@
       <c r="A113" s="11" t="n"/>
       <c r="B113" s="11" t="n"/>
       <c r="C113" s="11" t="n"/>
-      <c r="D113" s="22">
+      <c r="D113" s="23">
         <f>IF(A113="","",IFERROR(VLOOKUP(A113,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3508,7 +4426,7 @@
       <c r="A114" s="11" t="n"/>
       <c r="B114" s="11" t="n"/>
       <c r="C114" s="11" t="n"/>
-      <c r="D114" s="22">
+      <c r="D114" s="23">
         <f>IF(A114="","",IFERROR(VLOOKUP(A114,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3527,7 +4445,7 @@
       <c r="A115" s="11" t="n"/>
       <c r="B115" s="11" t="n"/>
       <c r="C115" s="11" t="n"/>
-      <c r="D115" s="22">
+      <c r="D115" s="23">
         <f>IF(A115="","",IFERROR(VLOOKUP(A115,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3546,7 +4464,7 @@
       <c r="A116" s="11" t="n"/>
       <c r="B116" s="11" t="n"/>
       <c r="C116" s="11" t="n"/>
-      <c r="D116" s="22">
+      <c r="D116" s="23">
         <f>IF(A116="","",IFERROR(VLOOKUP(A116,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3565,7 +4483,7 @@
       <c r="A117" s="11" t="n"/>
       <c r="B117" s="11" t="n"/>
       <c r="C117" s="11" t="n"/>
-      <c r="D117" s="22">
+      <c r="D117" s="23">
         <f>IF(A117="","",IFERROR(VLOOKUP(A117,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3584,7 +4502,7 @@
       <c r="A118" s="11" t="n"/>
       <c r="B118" s="11" t="n"/>
       <c r="C118" s="11" t="n"/>
-      <c r="D118" s="22">
+      <c r="D118" s="23">
         <f>IF(A118="","",IFERROR(VLOOKUP(A118,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3603,7 +4521,7 @@
       <c r="A119" s="11" t="n"/>
       <c r="B119" s="11" t="n"/>
       <c r="C119" s="11" t="n"/>
-      <c r="D119" s="22">
+      <c r="D119" s="23">
         <f>IF(A119="","",IFERROR(VLOOKUP(A119,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3622,7 +4540,7 @@
       <c r="A120" s="11" t="n"/>
       <c r="B120" s="11" t="n"/>
       <c r="C120" s="11" t="n"/>
-      <c r="D120" s="22">
+      <c r="D120" s="23">
         <f>IF(A120="","",IFERROR(VLOOKUP(A120,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3641,7 +4559,7 @@
       <c r="A121" s="11" t="n"/>
       <c r="B121" s="11" t="n"/>
       <c r="C121" s="11" t="n"/>
-      <c r="D121" s="22">
+      <c r="D121" s="23">
         <f>IF(A121="","",IFERROR(VLOOKUP(A121,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3660,7 +4578,7 @@
       <c r="A122" s="11" t="n"/>
       <c r="B122" s="11" t="n"/>
       <c r="C122" s="11" t="n"/>
-      <c r="D122" s="22">
+      <c r="D122" s="23">
         <f>IF(A122="","",IFERROR(VLOOKUP(A122,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3679,7 +4597,7 @@
       <c r="A123" s="11" t="n"/>
       <c r="B123" s="11" t="n"/>
       <c r="C123" s="11" t="n"/>
-      <c r="D123" s="22">
+      <c r="D123" s="23">
         <f>IF(A123="","",IFERROR(VLOOKUP(A123,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3698,7 +4616,7 @@
       <c r="A124" s="11" t="n"/>
       <c r="B124" s="11" t="n"/>
       <c r="C124" s="11" t="n"/>
-      <c r="D124" s="22">
+      <c r="D124" s="23">
         <f>IF(A124="","",IFERROR(VLOOKUP(A124,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3717,7 +4635,7 @@
       <c r="A125" s="11" t="n"/>
       <c r="B125" s="11" t="n"/>
       <c r="C125" s="11" t="n"/>
-      <c r="D125" s="22">
+      <c r="D125" s="23">
         <f>IF(A125="","",IFERROR(VLOOKUP(A125,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3736,7 +4654,7 @@
       <c r="A126" s="11" t="n"/>
       <c r="B126" s="11" t="n"/>
       <c r="C126" s="11" t="n"/>
-      <c r="D126" s="22">
+      <c r="D126" s="23">
         <f>IF(A126="","",IFERROR(VLOOKUP(A126,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3755,7 +4673,7 @@
       <c r="A127" s="11" t="n"/>
       <c r="B127" s="11" t="n"/>
       <c r="C127" s="11" t="n"/>
-      <c r="D127" s="22">
+      <c r="D127" s="23">
         <f>IF(A127="","",IFERROR(VLOOKUP(A127,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3774,7 +4692,7 @@
       <c r="A128" s="11" t="n"/>
       <c r="B128" s="11" t="n"/>
       <c r="C128" s="11" t="n"/>
-      <c r="D128" s="22">
+      <c r="D128" s="23">
         <f>IF(A128="","",IFERROR(VLOOKUP(A128,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3793,7 +4711,7 @@
       <c r="A129" s="11" t="n"/>
       <c r="B129" s="11" t="n"/>
       <c r="C129" s="11" t="n"/>
-      <c r="D129" s="22">
+      <c r="D129" s="23">
         <f>IF(A129="","",IFERROR(VLOOKUP(A129,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3812,7 +4730,7 @@
       <c r="A130" s="11" t="n"/>
       <c r="B130" s="11" t="n"/>
       <c r="C130" s="11" t="n"/>
-      <c r="D130" s="22">
+      <c r="D130" s="23">
         <f>IF(A130="","",IFERROR(VLOOKUP(A130,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3831,7 +4749,7 @@
       <c r="A131" s="11" t="n"/>
       <c r="B131" s="11" t="n"/>
       <c r="C131" s="11" t="n"/>
-      <c r="D131" s="22">
+      <c r="D131" s="23">
         <f>IF(A131="","",IFERROR(VLOOKUP(A131,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3850,7 +4768,7 @@
       <c r="A132" s="11" t="n"/>
       <c r="B132" s="11" t="n"/>
       <c r="C132" s="11" t="n"/>
-      <c r="D132" s="22">
+      <c r="D132" s="23">
         <f>IF(A132="","",IFERROR(VLOOKUP(A132,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3869,7 +4787,7 @@
       <c r="A133" s="11" t="n"/>
       <c r="B133" s="11" t="n"/>
       <c r="C133" s="11" t="n"/>
-      <c r="D133" s="22">
+      <c r="D133" s="23">
         <f>IF(A133="","",IFERROR(VLOOKUP(A133,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3888,7 +4806,7 @@
       <c r="A134" s="11" t="n"/>
       <c r="B134" s="11" t="n"/>
       <c r="C134" s="11" t="n"/>
-      <c r="D134" s="22">
+      <c r="D134" s="23">
         <f>IF(A134="","",IFERROR(VLOOKUP(A134,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3907,7 +4825,7 @@
       <c r="A135" s="11" t="n"/>
       <c r="B135" s="11" t="n"/>
       <c r="C135" s="11" t="n"/>
-      <c r="D135" s="22">
+      <c r="D135" s="23">
         <f>IF(A135="","",IFERROR(VLOOKUP(A135,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3926,7 +4844,7 @@
       <c r="A136" s="11" t="n"/>
       <c r="B136" s="11" t="n"/>
       <c r="C136" s="11" t="n"/>
-      <c r="D136" s="22">
+      <c r="D136" s="23">
         <f>IF(A136="","",IFERROR(VLOOKUP(A136,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3945,7 +4863,7 @@
       <c r="A137" s="11" t="n"/>
       <c r="B137" s="11" t="n"/>
       <c r="C137" s="11" t="n"/>
-      <c r="D137" s="22">
+      <c r="D137" s="23">
         <f>IF(A137="","",IFERROR(VLOOKUP(A137,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3964,7 +4882,7 @@
       <c r="A138" s="11" t="n"/>
       <c r="B138" s="11" t="n"/>
       <c r="C138" s="11" t="n"/>
-      <c r="D138" s="22">
+      <c r="D138" s="23">
         <f>IF(A138="","",IFERROR(VLOOKUP(A138,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -3983,7 +4901,7 @@
       <c r="A139" s="11" t="n"/>
       <c r="B139" s="11" t="n"/>
       <c r="C139" s="11" t="n"/>
-      <c r="D139" s="22">
+      <c r="D139" s="23">
         <f>IF(A139="","",IFERROR(VLOOKUP(A139,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4002,7 +4920,7 @@
       <c r="A140" s="11" t="n"/>
       <c r="B140" s="11" t="n"/>
       <c r="C140" s="11" t="n"/>
-      <c r="D140" s="22">
+      <c r="D140" s="23">
         <f>IF(A140="","",IFERROR(VLOOKUP(A140,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4021,7 +4939,7 @@
       <c r="A141" s="11" t="n"/>
       <c r="B141" s="11" t="n"/>
       <c r="C141" s="11" t="n"/>
-      <c r="D141" s="22">
+      <c r="D141" s="23">
         <f>IF(A141="","",IFERROR(VLOOKUP(A141,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4040,7 +4958,7 @@
       <c r="A142" s="11" t="n"/>
       <c r="B142" s="11" t="n"/>
       <c r="C142" s="11" t="n"/>
-      <c r="D142" s="22">
+      <c r="D142" s="23">
         <f>IF(A142="","",IFERROR(VLOOKUP(A142,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4059,7 +4977,7 @@
       <c r="A143" s="11" t="n"/>
       <c r="B143" s="11" t="n"/>
       <c r="C143" s="11" t="n"/>
-      <c r="D143" s="22">
+      <c r="D143" s="23">
         <f>IF(A143="","",IFERROR(VLOOKUP(A143,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4078,7 +4996,7 @@
       <c r="A144" s="11" t="n"/>
       <c r="B144" s="11" t="n"/>
       <c r="C144" s="11" t="n"/>
-      <c r="D144" s="22">
+      <c r="D144" s="23">
         <f>IF(A144="","",IFERROR(VLOOKUP(A144,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4097,7 +5015,7 @@
       <c r="A145" s="11" t="n"/>
       <c r="B145" s="11" t="n"/>
       <c r="C145" s="11" t="n"/>
-      <c r="D145" s="22">
+      <c r="D145" s="23">
         <f>IF(A145="","",IFERROR(VLOOKUP(A145,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4116,7 +5034,7 @@
       <c r="A146" s="11" t="n"/>
       <c r="B146" s="11" t="n"/>
       <c r="C146" s="11" t="n"/>
-      <c r="D146" s="22">
+      <c r="D146" s="23">
         <f>IF(A146="","",IFERROR(VLOOKUP(A146,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4135,7 +5053,7 @@
       <c r="A147" s="11" t="n"/>
       <c r="B147" s="11" t="n"/>
       <c r="C147" s="11" t="n"/>
-      <c r="D147" s="22">
+      <c r="D147" s="23">
         <f>IF(A147="","",IFERROR(VLOOKUP(A147,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4154,7 +5072,7 @@
       <c r="A148" s="11" t="n"/>
       <c r="B148" s="11" t="n"/>
       <c r="C148" s="11" t="n"/>
-      <c r="D148" s="22">
+      <c r="D148" s="23">
         <f>IF(A148="","",IFERROR(VLOOKUP(A148,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4173,7 +5091,7 @@
       <c r="A149" s="11" t="n"/>
       <c r="B149" s="11" t="n"/>
       <c r="C149" s="11" t="n"/>
-      <c r="D149" s="22">
+      <c r="D149" s="23">
         <f>IF(A149="","",IFERROR(VLOOKUP(A149,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4192,7 +5110,7 @@
       <c r="A150" s="11" t="n"/>
       <c r="B150" s="11" t="n"/>
       <c r="C150" s="11" t="n"/>
-      <c r="D150" s="22">
+      <c r="D150" s="23">
         <f>IF(A150="","",IFERROR(VLOOKUP(A150,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4211,7 +5129,7 @@
       <c r="A151" s="11" t="n"/>
       <c r="B151" s="11" t="n"/>
       <c r="C151" s="11" t="n"/>
-      <c r="D151" s="22">
+      <c r="D151" s="23">
         <f>IF(A151="","",IFERROR(VLOOKUP(A151,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4230,7 +5148,7 @@
       <c r="A152" s="11" t="n"/>
       <c r="B152" s="11" t="n"/>
       <c r="C152" s="11" t="n"/>
-      <c r="D152" s="22">
+      <c r="D152" s="23">
         <f>IF(A152="","",IFERROR(VLOOKUP(A152,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4249,7 +5167,7 @@
       <c r="A153" s="11" t="n"/>
       <c r="B153" s="11" t="n"/>
       <c r="C153" s="11" t="n"/>
-      <c r="D153" s="22">
+      <c r="D153" s="23">
         <f>IF(A153="","",IFERROR(VLOOKUP(A153,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4268,7 +5186,7 @@
       <c r="A154" s="11" t="n"/>
       <c r="B154" s="11" t="n"/>
       <c r="C154" s="11" t="n"/>
-      <c r="D154" s="22">
+      <c r="D154" s="23">
         <f>IF(A154="","",IFERROR(VLOOKUP(A154,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4287,7 +5205,7 @@
       <c r="A155" s="11" t="n"/>
       <c r="B155" s="11" t="n"/>
       <c r="C155" s="11" t="n"/>
-      <c r="D155" s="22">
+      <c r="D155" s="23">
         <f>IF(A155="","",IFERROR(VLOOKUP(A155,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4306,7 +5224,7 @@
       <c r="A156" s="11" t="n"/>
       <c r="B156" s="11" t="n"/>
       <c r="C156" s="11" t="n"/>
-      <c r="D156" s="22">
+      <c r="D156" s="23">
         <f>IF(A156="","",IFERROR(VLOOKUP(A156,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4325,7 +5243,7 @@
       <c r="A157" s="11" t="n"/>
       <c r="B157" s="11" t="n"/>
       <c r="C157" s="11" t="n"/>
-      <c r="D157" s="22">
+      <c r="D157" s="23">
         <f>IF(A157="","",IFERROR(VLOOKUP(A157,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4344,7 +5262,7 @@
       <c r="A158" s="11" t="n"/>
       <c r="B158" s="11" t="n"/>
       <c r="C158" s="11" t="n"/>
-      <c r="D158" s="22">
+      <c r="D158" s="23">
         <f>IF(A158="","",IFERROR(VLOOKUP(A158,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4363,7 +5281,7 @@
       <c r="A159" s="11" t="n"/>
       <c r="B159" s="11" t="n"/>
       <c r="C159" s="11" t="n"/>
-      <c r="D159" s="22">
+      <c r="D159" s="23">
         <f>IF(A159="","",IFERROR(VLOOKUP(A159,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4382,7 +5300,7 @@
       <c r="A160" s="11" t="n"/>
       <c r="B160" s="11" t="n"/>
       <c r="C160" s="11" t="n"/>
-      <c r="D160" s="22">
+      <c r="D160" s="23">
         <f>IF(A160="","",IFERROR(VLOOKUP(A160,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4401,7 +5319,7 @@
       <c r="A161" s="11" t="n"/>
       <c r="B161" s="11" t="n"/>
       <c r="C161" s="11" t="n"/>
-      <c r="D161" s="22">
+      <c r="D161" s="23">
         <f>IF(A161="","",IFERROR(VLOOKUP(A161,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4420,7 +5338,7 @@
       <c r="A162" s="11" t="n"/>
       <c r="B162" s="11" t="n"/>
       <c r="C162" s="11" t="n"/>
-      <c r="D162" s="22">
+      <c r="D162" s="23">
         <f>IF(A162="","",IFERROR(VLOOKUP(A162,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4439,7 +5357,7 @@
       <c r="A163" s="11" t="n"/>
       <c r="B163" s="11" t="n"/>
       <c r="C163" s="11" t="n"/>
-      <c r="D163" s="22">
+      <c r="D163" s="23">
         <f>IF(A163="","",IFERROR(VLOOKUP(A163,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4458,7 +5376,7 @@
       <c r="A164" s="11" t="n"/>
       <c r="B164" s="11" t="n"/>
       <c r="C164" s="11" t="n"/>
-      <c r="D164" s="22">
+      <c r="D164" s="23">
         <f>IF(A164="","",IFERROR(VLOOKUP(A164,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4477,7 +5395,7 @@
       <c r="A165" s="11" t="n"/>
       <c r="B165" s="11" t="n"/>
       <c r="C165" s="11" t="n"/>
-      <c r="D165" s="22">
+      <c r="D165" s="23">
         <f>IF(A165="","",IFERROR(VLOOKUP(A165,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4496,7 +5414,7 @@
       <c r="A166" s="11" t="n"/>
       <c r="B166" s="11" t="n"/>
       <c r="C166" s="11" t="n"/>
-      <c r="D166" s="22">
+      <c r="D166" s="23">
         <f>IF(A166="","",IFERROR(VLOOKUP(A166,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4515,7 +5433,7 @@
       <c r="A167" s="11" t="n"/>
       <c r="B167" s="11" t="n"/>
       <c r="C167" s="11" t="n"/>
-      <c r="D167" s="22">
+      <c r="D167" s="23">
         <f>IF(A167="","",IFERROR(VLOOKUP(A167,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4534,7 +5452,7 @@
       <c r="A168" s="11" t="n"/>
       <c r="B168" s="11" t="n"/>
       <c r="C168" s="11" t="n"/>
-      <c r="D168" s="22">
+      <c r="D168" s="23">
         <f>IF(A168="","",IFERROR(VLOOKUP(A168,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4553,7 +5471,7 @@
       <c r="A169" s="11" t="n"/>
       <c r="B169" s="11" t="n"/>
       <c r="C169" s="11" t="n"/>
-      <c r="D169" s="22">
+      <c r="D169" s="23">
         <f>IF(A169="","",IFERROR(VLOOKUP(A169,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4572,7 +5490,7 @@
       <c r="A170" s="11" t="n"/>
       <c r="B170" s="11" t="n"/>
       <c r="C170" s="11" t="n"/>
-      <c r="D170" s="22">
+      <c r="D170" s="23">
         <f>IF(A170="","",IFERROR(VLOOKUP(A170,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4591,7 +5509,7 @@
       <c r="A171" s="11" t="n"/>
       <c r="B171" s="11" t="n"/>
       <c r="C171" s="11" t="n"/>
-      <c r="D171" s="22">
+      <c r="D171" s="23">
         <f>IF(A171="","",IFERROR(VLOOKUP(A171,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4610,7 +5528,7 @@
       <c r="A172" s="11" t="n"/>
       <c r="B172" s="11" t="n"/>
       <c r="C172" s="11" t="n"/>
-      <c r="D172" s="22">
+      <c r="D172" s="23">
         <f>IF(A172="","",IFERROR(VLOOKUP(A172,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4629,7 +5547,7 @@
       <c r="A173" s="11" t="n"/>
       <c r="B173" s="11" t="n"/>
       <c r="C173" s="11" t="n"/>
-      <c r="D173" s="22">
+      <c r="D173" s="23">
         <f>IF(A173="","",IFERROR(VLOOKUP(A173,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4648,7 +5566,7 @@
       <c r="A174" s="11" t="n"/>
       <c r="B174" s="11" t="n"/>
       <c r="C174" s="11" t="n"/>
-      <c r="D174" s="22">
+      <c r="D174" s="23">
         <f>IF(A174="","",IFERROR(VLOOKUP(A174,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4667,7 +5585,7 @@
       <c r="A175" s="11" t="n"/>
       <c r="B175" s="11" t="n"/>
       <c r="C175" s="11" t="n"/>
-      <c r="D175" s="22">
+      <c r="D175" s="23">
         <f>IF(A175="","",IFERROR(VLOOKUP(A175,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4686,7 +5604,7 @@
       <c r="A176" s="11" t="n"/>
       <c r="B176" s="11" t="n"/>
       <c r="C176" s="11" t="n"/>
-      <c r="D176" s="22">
+      <c r="D176" s="23">
         <f>IF(A176="","",IFERROR(VLOOKUP(A176,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4705,7 +5623,7 @@
       <c r="A177" s="11" t="n"/>
       <c r="B177" s="11" t="n"/>
       <c r="C177" s="11" t="n"/>
-      <c r="D177" s="22">
+      <c r="D177" s="23">
         <f>IF(A177="","",IFERROR(VLOOKUP(A177,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4724,7 +5642,7 @@
       <c r="A178" s="11" t="n"/>
       <c r="B178" s="11" t="n"/>
       <c r="C178" s="11" t="n"/>
-      <c r="D178" s="22">
+      <c r="D178" s="23">
         <f>IF(A178="","",IFERROR(VLOOKUP(A178,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4743,7 +5661,7 @@
       <c r="A179" s="11" t="n"/>
       <c r="B179" s="11" t="n"/>
       <c r="C179" s="11" t="n"/>
-      <c r="D179" s="22">
+      <c r="D179" s="23">
         <f>IF(A179="","",IFERROR(VLOOKUP(A179,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4762,7 +5680,7 @@
       <c r="A180" s="11" t="n"/>
       <c r="B180" s="11" t="n"/>
       <c r="C180" s="11" t="n"/>
-      <c r="D180" s="22">
+      <c r="D180" s="23">
         <f>IF(A180="","",IFERROR(VLOOKUP(A180,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4781,7 +5699,7 @@
       <c r="A181" s="11" t="n"/>
       <c r="B181" s="11" t="n"/>
       <c r="C181" s="11" t="n"/>
-      <c r="D181" s="22">
+      <c r="D181" s="23">
         <f>IF(A181="","",IFERROR(VLOOKUP(A181,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4800,7 +5718,7 @@
       <c r="A182" s="11" t="n"/>
       <c r="B182" s="11" t="n"/>
       <c r="C182" s="11" t="n"/>
-      <c r="D182" s="22">
+      <c r="D182" s="23">
         <f>IF(A182="","",IFERROR(VLOOKUP(A182,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4819,7 +5737,7 @@
       <c r="A183" s="11" t="n"/>
       <c r="B183" s="11" t="n"/>
       <c r="C183" s="11" t="n"/>
-      <c r="D183" s="22">
+      <c r="D183" s="23">
         <f>IF(A183="","",IFERROR(VLOOKUP(A183,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4838,7 +5756,7 @@
       <c r="A184" s="11" t="n"/>
       <c r="B184" s="11" t="n"/>
       <c r="C184" s="11" t="n"/>
-      <c r="D184" s="22">
+      <c r="D184" s="23">
         <f>IF(A184="","",IFERROR(VLOOKUP(A184,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4857,7 +5775,7 @@
       <c r="A185" s="11" t="n"/>
       <c r="B185" s="11" t="n"/>
       <c r="C185" s="11" t="n"/>
-      <c r="D185" s="22">
+      <c r="D185" s="23">
         <f>IF(A185="","",IFERROR(VLOOKUP(A185,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4876,7 +5794,7 @@
       <c r="A186" s="11" t="n"/>
       <c r="B186" s="11" t="n"/>
       <c r="C186" s="11" t="n"/>
-      <c r="D186" s="22">
+      <c r="D186" s="23">
         <f>IF(A186="","",IFERROR(VLOOKUP(A186,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4895,7 +5813,7 @@
       <c r="A187" s="11" t="n"/>
       <c r="B187" s="11" t="n"/>
       <c r="C187" s="11" t="n"/>
-      <c r="D187" s="22">
+      <c r="D187" s="23">
         <f>IF(A187="","",IFERROR(VLOOKUP(A187,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4914,7 +5832,7 @@
       <c r="A188" s="11" t="n"/>
       <c r="B188" s="11" t="n"/>
       <c r="C188" s="11" t="n"/>
-      <c r="D188" s="22">
+      <c r="D188" s="23">
         <f>IF(A188="","",IFERROR(VLOOKUP(A188,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4933,7 +5851,7 @@
       <c r="A189" s="11" t="n"/>
       <c r="B189" s="11" t="n"/>
       <c r="C189" s="11" t="n"/>
-      <c r="D189" s="22">
+      <c r="D189" s="23">
         <f>IF(A189="","",IFERROR(VLOOKUP(A189,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4952,7 +5870,7 @@
       <c r="A190" s="11" t="n"/>
       <c r="B190" s="11" t="n"/>
       <c r="C190" s="11" t="n"/>
-      <c r="D190" s="22">
+      <c r="D190" s="23">
         <f>IF(A190="","",IFERROR(VLOOKUP(A190,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4971,7 +5889,7 @@
       <c r="A191" s="11" t="n"/>
       <c r="B191" s="11" t="n"/>
       <c r="C191" s="11" t="n"/>
-      <c r="D191" s="22">
+      <c r="D191" s="23">
         <f>IF(A191="","",IFERROR(VLOOKUP(A191,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -4990,7 +5908,7 @@
       <c r="A192" s="11" t="n"/>
       <c r="B192" s="11" t="n"/>
       <c r="C192" s="11" t="n"/>
-      <c r="D192" s="22">
+      <c r="D192" s="23">
         <f>IF(A192="","",IFERROR(VLOOKUP(A192,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5009,7 +5927,7 @@
       <c r="A193" s="11" t="n"/>
       <c r="B193" s="11" t="n"/>
       <c r="C193" s="11" t="n"/>
-      <c r="D193" s="22">
+      <c r="D193" s="23">
         <f>IF(A193="","",IFERROR(VLOOKUP(A193,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5028,7 +5946,7 @@
       <c r="A194" s="11" t="n"/>
       <c r="B194" s="11" t="n"/>
       <c r="C194" s="11" t="n"/>
-      <c r="D194" s="22">
+      <c r="D194" s="23">
         <f>IF(A194="","",IFERROR(VLOOKUP(A194,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5047,7 +5965,7 @@
       <c r="A195" s="11" t="n"/>
       <c r="B195" s="11" t="n"/>
       <c r="C195" s="11" t="n"/>
-      <c r="D195" s="22">
+      <c r="D195" s="23">
         <f>IF(A195="","",IFERROR(VLOOKUP(A195,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5066,7 +5984,7 @@
       <c r="A196" s="11" t="n"/>
       <c r="B196" s="11" t="n"/>
       <c r="C196" s="11" t="n"/>
-      <c r="D196" s="22">
+      <c r="D196" s="23">
         <f>IF(A196="","",IFERROR(VLOOKUP(A196,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5085,7 +6003,7 @@
       <c r="A197" s="11" t="n"/>
       <c r="B197" s="11" t="n"/>
       <c r="C197" s="11" t="n"/>
-      <c r="D197" s="22">
+      <c r="D197" s="23">
         <f>IF(A197="","",IFERROR(VLOOKUP(A197,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5104,7 +6022,7 @@
       <c r="A198" s="11" t="n"/>
       <c r="B198" s="11" t="n"/>
       <c r="C198" s="11" t="n"/>
-      <c r="D198" s="22">
+      <c r="D198" s="23">
         <f>IF(A198="","",IFERROR(VLOOKUP(A198,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5123,7 +6041,7 @@
       <c r="A199" s="11" t="n"/>
       <c r="B199" s="11" t="n"/>
       <c r="C199" s="11" t="n"/>
-      <c r="D199" s="22">
+      <c r="D199" s="23">
         <f>IF(A199="","",IFERROR(VLOOKUP(A199,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5142,7 +6060,7 @@
       <c r="A200" s="11" t="n"/>
       <c r="B200" s="11" t="n"/>
       <c r="C200" s="11" t="n"/>
-      <c r="D200" s="22">
+      <c r="D200" s="23">
         <f>IF(A200="","",IFERROR(VLOOKUP(A200,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5161,7 +6079,7 @@
       <c r="A201" s="11" t="n"/>
       <c r="B201" s="11" t="n"/>
       <c r="C201" s="11" t="n"/>
-      <c r="D201" s="22">
+      <c r="D201" s="23">
         <f>IF(A201="","",IFERROR(VLOOKUP(A201,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5180,7 +6098,7 @@
       <c r="A202" s="11" t="n"/>
       <c r="B202" s="11" t="n"/>
       <c r="C202" s="11" t="n"/>
-      <c r="D202" s="22">
+      <c r="D202" s="23">
         <f>IF(A202="","",IFERROR(VLOOKUP(A202,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5199,7 +6117,7 @@
       <c r="A203" s="11" t="n"/>
       <c r="B203" s="11" t="n"/>
       <c r="C203" s="11" t="n"/>
-      <c r="D203" s="22">
+      <c r="D203" s="23">
         <f>IF(A203="","",IFERROR(VLOOKUP(A203,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5218,7 +6136,7 @@
       <c r="A204" s="11" t="n"/>
       <c r="B204" s="11" t="n"/>
       <c r="C204" s="11" t="n"/>
-      <c r="D204" s="22">
+      <c r="D204" s="23">
         <f>IF(A204="","",IFERROR(VLOOKUP(A204,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5237,7 +6155,7 @@
       <c r="A205" s="11" t="n"/>
       <c r="B205" s="11" t="n"/>
       <c r="C205" s="11" t="n"/>
-      <c r="D205" s="22">
+      <c r="D205" s="23">
         <f>IF(A205="","",IFERROR(VLOOKUP(A205,'صورت وضعیت پروژه'!$B$9:$G$48,2,0),"؟ آیتم پیدا نشد"))</f>
         <v/>
       </c>
@@ -5261,83 +6179,90 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>راهنمای پر کردن فایل</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>۱. در برگهٔ «صورت وضعیت پروژه» فقط خانه‌های کرم‌رنگ را پر کنید؛ ستون «مبلغ» خودکار حساب می‌شود.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>۲. ردیف‌های ۱ تا ۳۰ آیتم‌های اصلی قرارداد و ردیف‌های «مازاد بر قرارداد (n)» کارهای اضافه‌اند. ردیف خالی وارد نمی‌شود.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>۳. «نوع»: فروش / تأمین (بدون بیمه) — نصب (مشمول بیمهٔ ۱۶٫۶۷٪) — سایر. اگر خالی بماند از روی شرح حدس زده می‌شود.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>۴. «فی» و «مبلغ» به ریال. «مقدار» می‌تواند اعشاری باشد (مثلاً 249.89).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>۵. «تخفیف»: مبلغ کل تخفیف قرارداد به ریال (اختیاری). درصد تخفیف خودکار از آن حساب می‌شود.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>۶. برگهٔ «ریزمتر» اختیاری است: شمارهٔ آیتم (همان ستون اول برگهٔ قبل، مثل 3 یا «مازاد بر قرارداد (1)»)، شمارهٔ صورت وضعیت، تاریخ شمسی و مقدار انجام‌شده.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">   اگر شمارهٔ صورت وضعیت را «قطعی» بنویسید، آن ردیف‌ها صورت وضعیت بعدی و قطعی می‌شوند.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>۷. در LifeOS: پروژه › اطلاعات مالی › آیتم‌های قرارداد › «📥 ورود از اکسل» و همین فایل را انتخاب کنید.</t>
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>برگهٔ «نمونهٔ پرشده» فقط برای دیدن است و هیچ‌وقت وارد نمی‌شود.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>۷. در LifeOS: پروژه › اطلاعات مالی › آیتم‌های قرارداد › «📥 ورود از اکسل» و همین فایل را انتخاب کنید.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>نام برگه‌ها و عنوان ستون‌ها را تغییر ندهید؛ ستون‌ها از روی عنوانشان پیدا می‌شوند.</t>
         </is>

</xml_diff>